<commit_message>
feat: improve layout spacing, landing page, and interactive pipeline simulation stages
</commit_message>
<xml_diff>
--- a/samples/sample_questionnaire.xlsx
+++ b/samples/sample_questionnaire.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +25,22 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A2D5C"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +55,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,28 +428,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="65" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Response</t>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
         </is>
       </c>
     </row>
@@ -442,111 +457,406 @@
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Do you encrypt data at rest?</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Do you support SAML SSO and multi-factor authentication?</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Do you encrypt data in transit?</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Are you SOC 2 Type II certified?</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Do you support customer-managed encryption keys (BYOK)?</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Are you HIPAA certified?</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>What is your MFA policy?</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Where is customer data stored?</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Do you support SSO via SAML or OIDC?</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>What is your incident response notification SLA?</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>How do you handle vulnerability management?</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
         <v>7</v>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>How long are backups retained?</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Do you perform regular penetration testing?</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
         <v>8</v>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Do you guarantee zero breaches?</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>What is your uptime SLA?</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
         <v>9</v>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>What is your favorite color?</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Describe your disaster recovery capabilities.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
         <v>10</v>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Do you support customer-managed encryption keys?</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>What logging and monitoring do you provide?</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Technical</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Are you SOC 2 Type II certified?</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Certification</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Are you ISO 27001 certified?</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Certification</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Are you HIPAA certified?</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Certification</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Are you PCI DSS certified?</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Certification</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Are you FedRAMP authorized?</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Certification</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Where is customer data stored?</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Data Privacy</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>What is your data retention policy?</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Data Privacy</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Do you have a list of sub-processors?</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Data Privacy</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>How do you handle cross-border data transfers?</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Data Privacy</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Can we execute a Data Processing Agreement (DPA)?</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Data Privacy</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Do you guarantee zero security incidents?</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Will you indemnify us for data loss?</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>What are your SLA credits for downtime?</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Do you carry cyber liability insurance?</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Do you have a business continuity plan?</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>How do you train employees on security?</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>What is your incident response process?</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>